<commit_message>
20260610 complate Base V1.0
</commit_message>
<xml_diff>
--- a/burnerController_JXXY/20260330_烧嘴控制改造程序-点表.xlsx
+++ b/burnerController_JXXY/20260330_烧嘴控制改造程序-点表.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\codes\04-electricity\01-plc\江铜\burnerControler_JXT\burnerController_JXXY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B349EC95-C1BD-4C41-B3B9-CCCDA796619F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20ABDC59-709F-4F66-A4EF-4DB7F8450ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookPassword="EF03" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="990" windowWidth="13560" windowHeight="13725" activeTab="7" xr2:uid="{2BCBB78C-AFBE-4F13-8C2E-200396EF23E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{2BCBB78C-AFBE-4F13-8C2E-200396EF23E4}"/>
   </bookViews>
   <sheets>
     <sheet name="命名规范" sheetId="8" r:id="rId1"/>

</xml_diff>

<commit_message>
add Test sheet to excel
</commit_message>
<xml_diff>
--- a/burnerController_JXXY/20260330_烧嘴控制改造程序-点表.xlsx
+++ b/burnerController_JXXY/20260330_烧嘴控制改造程序-点表.xlsx
@@ -1,58 +1,72 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\codes\04-electricity\01-plc\江铜\burnerControler_JXT\burnerController_JXXY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\02-PLC项目\江西沸腾炉烧嘴程序改造\burnerController_JXXY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20ABDC59-709F-4F66-A4EF-4DB7F8450ED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <workbookProtection workbookPassword="EF03" lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D263828-DFB1-40EF-B1E0-02B05C273EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{2BCBB78C-AFBE-4F13-8C2E-200396EF23E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="622" activeTab="1" xr2:uid="{2BCBB78C-AFBE-4F13-8C2E-200396EF23E4}"/>
   </bookViews>
   <sheets>
     <sheet name="命名规范" sheetId="8" r:id="rId1"/>
-    <sheet name="端子1" sheetId="1" r:id="rId2"/>
-    <sheet name="符号表" sheetId="7" r:id="rId3"/>
-    <sheet name="通讯" sheetId="5" r:id="rId4"/>
-    <sheet name="符号模板" sheetId="9" r:id="rId5"/>
-    <sheet name="1英文命名" sheetId="11" r:id="rId6"/>
-    <sheet name="2命名后改地址" sheetId="12" r:id="rId7"/>
-    <sheet name="3符号地址校验" sheetId="13" r:id="rId8"/>
-    <sheet name="IO分配表" sheetId="14" r:id="rId9"/>
-    <sheet name="数据项" sheetId="6" r:id="rId10"/>
+    <sheet name="测试" sheetId="15" r:id="rId2"/>
+    <sheet name="端子1" sheetId="1" r:id="rId3"/>
+    <sheet name="符号表" sheetId="7" r:id="rId4"/>
+    <sheet name="通讯" sheetId="5" r:id="rId5"/>
+    <sheet name="符号模板" sheetId="9" r:id="rId6"/>
+    <sheet name="1英文命名" sheetId="11" r:id="rId7"/>
+    <sheet name="2命名后改地址" sheetId="12" r:id="rId8"/>
+    <sheet name="3符号地址校验" sheetId="13" r:id="rId9"/>
+    <sheet name="IO分配表" sheetId="14" r:id="rId10"/>
+    <sheet name="数据项" sheetId="6" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'1英文命名'!$C$1:$E$76</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'2命名后改地址'!$C$1:$E$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'3符号地址校验'!$E$1:$G$74</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">端子1!$C$1:$E$76</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">符号表!$C$1:$E$61</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'1英文命名'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'2命名后改地址'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'3符号地址校验'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">端子1!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">符号表!#REF!</definedName>
-    <definedName name="VW区" localSheetId="5">'1英文命名'!#REF!</definedName>
-    <definedName name="VW区" localSheetId="6">'2命名后改地址'!#REF!</definedName>
-    <definedName name="VW区" localSheetId="7">'3符号地址校验'!#REF!</definedName>
-    <definedName name="VW区" localSheetId="2">符号表!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'1英文命名'!$C$1:$E$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'2命名后改地址'!$C$1:$E$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'3符号地址校验'!$E$1:$G$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">端子1!$C$1:$E$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">符号表!$C$1:$E$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'1英文命名'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'2命名后改地址'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'3符号地址校验'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">端子1!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">符号表!#REF!</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">测试!$1:$1</definedName>
+    <definedName name="VW区" localSheetId="6">'1英文命名'!#REF!</definedName>
+    <definedName name="VW区" localSheetId="7">'2命名后改地址'!#REF!</definedName>
+    <definedName name="VW区" localSheetId="8">'3符号地址校验'!#REF!</definedName>
+    <definedName name="VW区" localSheetId="3">符号表!#REF!</definedName>
     <definedName name="VW区">端子1!#REF!</definedName>
-    <definedName name="V区" localSheetId="5">'1英文命名'!#REF!</definedName>
-    <definedName name="V区" localSheetId="6">'2命名后改地址'!#REF!</definedName>
-    <definedName name="V区" localSheetId="7">'3符号地址校验'!#REF!</definedName>
-    <definedName name="V区" localSheetId="2">符号表!#REF!</definedName>
+    <definedName name="V区" localSheetId="6">'1英文命名'!#REF!</definedName>
+    <definedName name="V区" localSheetId="7">'2命名后改地址'!#REF!</definedName>
+    <definedName name="V区" localSheetId="8">'3符号地址校验'!#REF!</definedName>
+    <definedName name="V区" localSheetId="3">符号表!#REF!</definedName>
     <definedName name="V区">端子1!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4588" uniqueCount="1737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4678" uniqueCount="1792">
   <si>
     <t>I</t>
   </si>
@@ -5603,6 +5617,203 @@
 12.故障报警</t>
     <phoneticPr fontId="21" type="noConversion"/>
   </si>
+  <si>
+    <t>操作步骤</t>
+  </si>
+  <si>
+    <t>预期结果</t>
+  </si>
+  <si>
+    <t>实测结果</t>
+  </si>
+  <si>
+    <t>☐ 通过</t>
+  </si>
+  <si>
+    <t>异常</t>
+  </si>
+  <si>
+    <t>检漏异常报警，并且无法开机，必须再次检漏，通过后才能开机。</t>
+  </si>
+  <si>
+    <t>检测通过</t>
+  </si>
+  <si>
+    <t>不能启动</t>
+  </si>
+  <si>
+    <t>吹扫</t>
+  </si>
+  <si>
+    <t>正常吹扫</t>
+  </si>
+  <si>
+    <t>点火准备</t>
+  </si>
+  <si>
+    <t>正常进入点火</t>
+  </si>
+  <si>
+    <t>高压放电，持续【打火时长】秒时间，火焰稳定超过2秒</t>
+  </si>
+  <si>
+    <t>点火成功，转入小火运行</t>
+  </si>
+  <si>
+    <t>高压放电打火结束，没建立火焰或火焰无法稳定【火焰建立时长】1秒以上，点火失败</t>
+  </si>
+  <si>
+    <t>报警：点火失败</t>
+  </si>
+  <si>
+    <t>火焰丢失</t>
+  </si>
+  <si>
+    <t>正常运行中，火焰丢失超过2【火焰丢失延时】秒，报警</t>
+  </si>
+  <si>
+    <t>报警：火焰丢失</t>
+  </si>
+  <si>
+    <t>主火运行</t>
+  </si>
+  <si>
+    <t>开启主火阀V2、安全阀V1</t>
+  </si>
+  <si>
+    <t>阀正常开启</t>
+  </si>
+  <si>
+    <t>温控启停</t>
+  </si>
+  <si>
+    <t>调节当前温度为超过停机温度</t>
+  </si>
+  <si>
+    <t>超过设定温度，关闭主火阀、安全阀</t>
+  </si>
+  <si>
+    <t>手动模式</t>
+  </si>
+  <si>
+    <t>手动模式按屏幕上增档、减档</t>
+  </si>
+  <si>
+    <t>档位随增减档而变动</t>
+  </si>
+  <si>
+    <t>自动模式</t>
+  </si>
+  <si>
+    <t>自动模式升降档由PID控制，改变当前温度，观察档位变化情况</t>
+  </si>
+  <si>
+    <t>随温度升高而降档</t>
+  </si>
+  <si>
+    <t>阶段升温</t>
+  </si>
+  <si>
+    <t>观察目标温度是否按照设定的温度变化</t>
+  </si>
+  <si>
+    <t>会变化</t>
+  </si>
+  <si>
+    <t>485通讯</t>
+  </si>
+  <si>
+    <t>能看到</t>
+  </si>
+  <si>
+    <t>本地_远程</t>
+  </si>
+  <si>
+    <t>本地_远程互斥</t>
+  </si>
+  <si>
+    <t>上电-检漏
+手动-检漏</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>V1灯亮，接通燃气低压开关
+V2灯亮，关闭燃气低压开关</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>在30秒内
+空气调节阀打开至吹扫位置
+燃气调节阀打开至20%</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>上电-调节阀检测
+手动-调节阀检测</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>V1灯亮，不接通燃气低压开关
+V2灯亮，燃气低压开关接能，不关闭</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>在30秒内
+1、空气调节阀没有打开至吹扫位置
+2、燃气调节阀没有打开至20%</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>HMI 空气调节阀 闪红灯
+HMI 燃气调节阀 闪红灯</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>上电-检测中启动
+手动-检测中启动</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>以上四步
+在进行检测中，按启动按钮</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>调节阀走到位，开始吹扫
+调节阀没走到位，达到限制时长30秒，开始吹扫</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>调节阀走到位，开始点火
+调节阀没走到位，达到限制时长30秒，开始点火</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>观察远程是否能正常看到设备状态
+故障状态、自动状态、启动状态、停止状态、远程状态
+空气调节阀开度、燃气调节阀开度、当前温度、当前档位、PID温度（阶段6）</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>切换本地远程旋钮
+操作 启动、停止、复位</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>正常</t>
+  </si>
+  <si>
+    <t>正常</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>类别</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
+  <si>
+    <t>项目</t>
+    <phoneticPr fontId="32" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -5613,7 +5824,7 @@
     <numFmt numFmtId="177" formatCode="0.0_ "/>
     <numFmt numFmtId="178" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <sz val="12"/>
       <name val="宋体"/>
@@ -5793,6 +6004,12 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5941,7 +6158,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6182,12 +6399,143 @@
     <xf numFmtId="0" fontId="31" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
     <cellStyle name="常规 4 2" xfId="1" xr:uid="{C97CC49E-8548-40A7-B373-8E3F8F01BD97}"/>
   </cellStyles>
-  <dxfs count="87">
+  <dxfs count="94">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="16"/>
+        <color auto="1"/>
+        <name val="宋体"/>
+        <charset val="134"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -8183,156 +8531,170 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BC6A3F09-E86C-49A8-B91A-E1B95FD203B0}" name="表8" displayName="表8" ref="A1:F21" totalsRowShown="0" headerRowDxfId="86" dataDxfId="84" headerRowBorderDxfId="85" tableBorderDxfId="83">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{BC6A3F09-E86C-49A8-B91A-E1B95FD203B0}" name="表8" displayName="表8" ref="A1:F21" totalsRowShown="0" headerRowDxfId="93" dataDxfId="91" headerRowBorderDxfId="92" tableBorderDxfId="90">
   <autoFilter ref="A1:F21" xr:uid="{31503A1A-3ED1-4869-9B93-C5ABFAC7625B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F21">
     <sortCondition ref="A1:A21"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="命名类型" dataDxfId="82"/>
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="名称" dataDxfId="81"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="代码" dataDxfId="80"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="存储区域" dataDxfId="79"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="示例" dataDxfId="78"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="说明" dataDxfId="77"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="命名类型" dataDxfId="89"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="名称" dataDxfId="88"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="代码" dataDxfId="87"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="存储区域" dataDxfId="86"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="示例" dataDxfId="85"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="说明" dataDxfId="84"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{03BE1E8C-8A27-4BF2-B5AD-7C3831A87FC9}" name="表37" displayName="表37" ref="A1:F21" totalsRowShown="0" headerRowDxfId="17" dataDxfId="15" headerRowBorderDxfId="16" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:F21" xr:uid="{E517E8B6-ADC0-4F95-930E-5AF82CCFF0B4}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="现场设备" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="地址" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="映射" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1100-000004000000}" name="符号" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1100-000005000000}" name="类型" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1100-000006000000}" name="备注" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF667D90-1EB1-4976-A8D5-70F378E47508}" name="表1" displayName="表1" ref="A1:F445" totalsRowShown="0" headerRowDxfId="76" dataDxfId="74" headerRowBorderDxfId="75" tableBorderDxfId="73">
-  <autoFilter ref="A1:F445" xr:uid="{EAEC5D8C-41E3-481D-8A3D-D139585DF349}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F445">
-    <sortCondition ref="B1:B445"/>
-  </sortState>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="存储区" dataDxfId="72"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="排序" dataDxfId="71"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="符号" dataDxfId="70"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="地址" dataDxfId="69"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="注释" dataDxfId="68"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="停电保持" dataDxfId="67"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{28DDED1F-1C4B-4D84-8FD0-826AE3C701E6}" name="表2" displayName="表2" ref="A1:E18" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A1:E18" xr:uid="{28DDED1F-1C4B-4D84-8FD0-826AE3C701E6}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{092C8F4C-750F-4A54-9775-0E878E7F692D}" name="类别" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{55E7343C-005A-47DD-BF51-A98FEB8687FA}" name="项目" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{E219FFED-DB05-4801-BA8C-E5182B5E135C}" name="操作步骤" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{37775F0D-5709-4D26-8B0D-3C61F165FF43}" name="预期结果" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{1DD79E4F-C3FB-4EA3-8CB8-5707D129384D}" name="实测结果" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{69D67C9D-053D-42BE-8EFD-926EE2DB3533}" name="表1_7" displayName="表1_7" ref="A1:F61" totalsRowShown="0" headerRowDxfId="66" dataDxfId="64" headerRowBorderDxfId="65" tableBorderDxfId="63">
-  <autoFilter ref="A1:F61" xr:uid="{81970FAC-CFE7-4A1D-A5CF-A2EACBF101FD}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F61">
-    <sortCondition ref="B1:B61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BF667D90-1EB1-4976-A8D5-70F378E47508}" name="表1" displayName="表1" ref="A1:F445" totalsRowShown="0" headerRowDxfId="83" dataDxfId="81" headerRowBorderDxfId="82" tableBorderDxfId="80">
+  <autoFilter ref="A1:F445" xr:uid="{EAEC5D8C-41E3-481D-8A3D-D139585DF349}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F445">
+    <sortCondition ref="B1:B445"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="存储区" dataDxfId="62"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="排序" dataDxfId="61">
-      <calculatedColumnFormula>VALUE(RIGHT(D2,LEN(D2)-LEN(A2)))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="符号" dataDxfId="60"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="地址" dataDxfId="59"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="注释" dataDxfId="58"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="停电保持" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="存储区" dataDxfId="79"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="排序" dataDxfId="78"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="符号" dataDxfId="77"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="地址" dataDxfId="76"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="注释" dataDxfId="75"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="停电保持" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="46" xr:uid="{819FCED7-92C0-4647-B4B4-EBF1A26CEDAE}" name="表46" displayName="表46" ref="B1:G17" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
-  <autoFilter ref="B1:G17" xr:uid="{94000AEE-EA2C-4D0D-8C4C-2ABB18A8C2A9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{69D67C9D-053D-42BE-8EFD-926EE2DB3533}" name="表1_7" displayName="表1_7" ref="A1:F61" totalsRowShown="0" headerRowDxfId="73" dataDxfId="71" headerRowBorderDxfId="72" tableBorderDxfId="70">
+  <autoFilter ref="A1:F61" xr:uid="{81970FAC-CFE7-4A1D-A5CF-A2EACBF101FD}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F61">
+    <sortCondition ref="B1:B61"/>
+  </sortState>
   <tableColumns count="6">
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="从站 HoldStar=500" dataDxfId="54"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="符号" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="从站 HoldStar=1500" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="注释" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Modbus主站地址" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="备注" dataDxfId="49"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="存储区" dataDxfId="69"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="排序" dataDxfId="68">
+      <calculatedColumnFormula>VALUE(RIGHT(D2,LEN(D2)-LEN(A2)))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="符号" dataDxfId="67"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="地址" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="注释" dataDxfId="65"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="停电保持" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{90352B38-6F74-4B30-9D89-B1BBC62CC6D9}" name="表15" displayName="表15" ref="A1:B3" totalsRowShown="0" headerRowDxfId="48" dataDxfId="46" headerRowBorderDxfId="47" tableBorderDxfId="45" totalsRowBorderDxfId="44">
-  <autoFilter ref="A1:B3" xr:uid="{2D618419-CC93-4748-AC73-50D15728A337}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="设备" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="缩写" dataDxfId="42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="46" xr:uid="{819FCED7-92C0-4647-B4B4-EBF1A26CEDAE}" name="表46" displayName="表46" ref="B1:G17" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+  <autoFilter ref="B1:G17" xr:uid="{94000AEE-EA2C-4D0D-8C4C-2ABB18A8C2A9}"/>
+  <tableColumns count="6">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="从站 HoldStar=500" dataDxfId="61"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="符号" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="从站 HoldStar=1500" dataDxfId="59"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="注释" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="Modbus主站地址" dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="备注" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{1B1EF626-8785-43D8-946F-EB282409C2A3}" name="表1_17" displayName="表1_17" ref="A1:F198" totalsRowShown="0" headerRowDxfId="41" dataDxfId="39" headerRowBorderDxfId="40" tableBorderDxfId="38">
-  <autoFilter ref="A1:F198" xr:uid="{3426D145-FA7C-4D4F-8D7A-5904FEA768E0}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F198">
-    <sortCondition ref="B1:B198"/>
-  </sortState>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="存储区" dataDxfId="37"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="排序" dataDxfId="36">
-      <calculatedColumnFormula>VALUE(RIGHT(D2,LEN(D2)-LEN(A2)))</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="符号" dataDxfId="35"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="地址" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="注释" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="停电保持" dataDxfId="32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{90352B38-6F74-4B30-9D89-B1BBC62CC6D9}" name="表15" displayName="表15" ref="A1:B3" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="51">
+  <autoFilter ref="A1:B3" xr:uid="{2D618419-CC93-4748-AC73-50D15728A337}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0900-000001000000}" name="设备" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0900-000002000000}" name="缩写" dataDxfId="49"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{4178DD1D-C394-4C90-A1E0-3503C781D35F}" name="表1_1718" displayName="表1_1718" ref="A1:F215" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28">
-  <autoFilter ref="A1:F215" xr:uid="{E8622A0D-4D7B-4CC8-BEC1-5B22455130E1}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A83:F215">
-    <sortCondition ref="B1:B215"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{1B1EF626-8785-43D8-946F-EB282409C2A3}" name="表1_17" displayName="表1_17" ref="A1:F198" totalsRowShown="0" headerRowDxfId="48" dataDxfId="46" headerRowBorderDxfId="47" tableBorderDxfId="45">
+  <autoFilter ref="A1:F198" xr:uid="{3426D145-FA7C-4D4F-8D7A-5904FEA768E0}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F198">
+    <sortCondition ref="B1:B198"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="存储区" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="排序" dataDxfId="26">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0B00-000001000000}" name="存储区" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0B00-000002000000}" name="排序" dataDxfId="43">
       <calculatedColumnFormula>VALUE(RIGHT(D2,LEN(D2)-LEN(A2)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="符号" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="地址" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="注释" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="停电保持" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0B00-000003000000}" name="符号" dataDxfId="42"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0B00-000004000000}" name="地址" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0B00-000005000000}" name="注释" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0B00-000006000000}" name="停电保持" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{D9EB2FB0-C2BE-41FC-99FB-6CD331B6BC5E}" name="符号表" displayName="符号表" ref="A1:G236" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18">
-  <autoFilter ref="A1:G236" xr:uid="{B3E6F695-5A5D-43F2-A4A9-C2D31569F3E9}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G223">
-    <sortCondition ref="F1:F223"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{4178DD1D-C394-4C90-A1E0-3503C781D35F}" name="表1_1718" displayName="表1_1718" ref="A1:F215" totalsRowShown="0" headerRowDxfId="38" dataDxfId="36" headerRowBorderDxfId="37" tableBorderDxfId="35">
+  <autoFilter ref="A1:F215" xr:uid="{E8622A0D-4D7B-4CC8-BEC1-5B22455130E1}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A83:F215">
+    <sortCondition ref="B1:B215"/>
   </sortState>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="存储区" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="排序" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0F00-000008000000}" name="间隔校验" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="符号长度" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="符号" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="地址" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="注释" dataDxfId="11"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0D00-000001000000}" name="存储区" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0D00-000002000000}" name="排序" dataDxfId="33">
+      <calculatedColumnFormula>VALUE(RIGHT(D2,LEN(D2)-LEN(A2)))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0D00-000003000000}" name="符号" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0D00-000004000000}" name="地址" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0D00-000005000000}" name="注释" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0D00-000006000000}" name="停电保持" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="37" xr:uid="{03BE1E8C-8A27-4BF2-B5AD-7C3831A87FC9}" name="表37" displayName="表37" ref="A1:F21" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
-  <autoFilter ref="A1:F21" xr:uid="{E517E8B6-ADC0-4F95-930E-5AF82CCFF0B4}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-1100-000001000000}" name="现场设备" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-1100-000002000000}" name="地址" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-1100-000003000000}" name="映射" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-1100-000004000000}" name="符号" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-1100-000005000000}" name="类型" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-1100-000006000000}" name="备注" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="36" xr:uid="{D9EB2FB0-C2BE-41FC-99FB-6CD331B6BC5E}" name="符号表" displayName="符号表" ref="A1:G236" totalsRowShown="0" headerRowDxfId="28" dataDxfId="26" headerRowBorderDxfId="27" tableBorderDxfId="25">
+  <autoFilter ref="A1:G236" xr:uid="{B3E6F695-5A5D-43F2-A4A9-C2D31569F3E9}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G223">
+    <sortCondition ref="F1:F223"/>
+  </sortState>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0F00-000001000000}" name="存储区" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0F00-000002000000}" name="排序" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0F00-000008000000}" name="间隔校验" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0F00-000007000000}" name="符号长度" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0F00-000003000000}" name="符号" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0F00-000004000000}" name="地址" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0F00-000005000000}" name="注释" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8950,6 +9312,426 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D43CC4C-71E3-46F9-8C94-C607BA6D0756}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="17.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="8" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20" style="42" customWidth="1"/>
+    <col min="5" max="5" width="6.625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="18.375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="58" customFormat="1" ht="24.95" customHeight="1">
+      <c r="A1" s="55" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B1" s="75" t="s">
+        <v>1726</v>
+      </c>
+      <c r="C1" s="75" t="s">
+        <v>1727</v>
+      </c>
+      <c r="D1" s="56" t="s">
+        <v>1535</v>
+      </c>
+      <c r="E1" s="57" t="s">
+        <v>1536</v>
+      </c>
+      <c r="F1" s="56" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A2" s="50" t="s">
+        <v>1537</v>
+      </c>
+      <c r="B2" s="51" t="s">
+        <v>1538</v>
+      </c>
+      <c r="C2" s="51" t="s">
+        <v>1516</v>
+      </c>
+      <c r="D2" s="59" t="s">
+        <v>1539</v>
+      </c>
+      <c r="E2" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A3" s="50" t="s">
+        <v>1567</v>
+      </c>
+      <c r="B3" s="51" t="s">
+        <v>1545</v>
+      </c>
+      <c r="C3" s="51" t="s">
+        <v>558</v>
+      </c>
+      <c r="D3" s="59" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E3" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F3" s="49" t="s">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A4" s="50" t="s">
+        <v>1568</v>
+      </c>
+      <c r="B4" s="51" t="s">
+        <v>1546</v>
+      </c>
+      <c r="C4" s="51" t="s">
+        <v>559</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>1046</v>
+      </c>
+      <c r="E4" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F4" s="49" t="s">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.5">
+      <c r="A5" s="50" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B5" s="51" t="s">
+        <v>1547</v>
+      </c>
+      <c r="C5" s="51" t="s">
+        <v>1552</v>
+      </c>
+      <c r="D5" s="59" t="s">
+        <v>811</v>
+      </c>
+      <c r="E5" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F5" s="74" t="s">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A6" s="50" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B6" s="51" t="s">
+        <v>1548</v>
+      </c>
+      <c r="C6" s="51" t="s">
+        <v>562</v>
+      </c>
+      <c r="D6" s="59" t="s">
+        <v>1047</v>
+      </c>
+      <c r="E6" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F6" s="46" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A7" s="50" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B7" s="51" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C7" s="51" t="s">
+        <v>563</v>
+      </c>
+      <c r="D7" s="59" t="s">
+        <v>815</v>
+      </c>
+      <c r="E7" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F7" s="46" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A8" s="50" t="s">
+        <v>1543</v>
+      </c>
+      <c r="B8" s="51" t="s">
+        <v>1550</v>
+      </c>
+      <c r="C8" s="51" t="s">
+        <v>818</v>
+      </c>
+      <c r="D8" s="59" t="s">
+        <v>817</v>
+      </c>
+      <c r="E8" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F8" s="46" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.5">
+      <c r="A9" s="50" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B9" s="51" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>564</v>
+      </c>
+      <c r="D9" s="59" t="s">
+        <v>820</v>
+      </c>
+      <c r="E9" s="52" t="s">
+        <v>1540</v>
+      </c>
+      <c r="F9" s="60" t="s">
+        <v>1566</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A10" s="76" t="s">
+        <v>1728</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>1562</v>
+      </c>
+      <c r="D10" s="48" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E10" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F10" s="46"/>
+    </row>
+    <row r="11" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A11" s="53" t="s">
+        <v>1564</v>
+      </c>
+      <c r="B11" s="46" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>571</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>1507</v>
+      </c>
+      <c r="E11" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F11" s="46"/>
+    </row>
+    <row r="12" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A12" s="53" t="s">
+        <v>1565</v>
+      </c>
+      <c r="B12" s="46" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>572</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>827</v>
+      </c>
+      <c r="E12" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F12" s="46"/>
+    </row>
+    <row r="13" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A13" s="53" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B13" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="46" t="s">
+        <v>573</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>829</v>
+      </c>
+      <c r="E13" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F13" s="46"/>
+    </row>
+    <row r="14" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A14" s="53" t="s">
+        <v>832</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>574</v>
+      </c>
+      <c r="D14" s="48" t="s">
+        <v>1480</v>
+      </c>
+      <c r="E14" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F14" s="46"/>
+    </row>
+    <row r="15" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A15" s="53" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>575</v>
+      </c>
+      <c r="D15" s="48" t="s">
+        <v>1481</v>
+      </c>
+      <c r="E15" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F15" s="46"/>
+    </row>
+    <row r="16" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A16" s="53" t="s">
+        <v>87</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>576</v>
+      </c>
+      <c r="D16" s="48" t="s">
+        <v>1482</v>
+      </c>
+      <c r="E16" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F16" s="46"/>
+    </row>
+    <row r="17" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A17" s="50" t="s">
+        <v>1560</v>
+      </c>
+      <c r="B17" s="51" t="s">
+        <v>97</v>
+      </c>
+      <c r="C17" s="46" t="s">
+        <v>577</v>
+      </c>
+      <c r="D17" s="59" t="s">
+        <v>836</v>
+      </c>
+      <c r="E17" s="54" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F17" s="51"/>
+    </row>
+    <row r="18" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A18" s="53" t="s">
+        <v>1573</v>
+      </c>
+      <c r="B18" s="46" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C18" s="46"/>
+      <c r="D18" s="48" t="s">
+        <v>1498</v>
+      </c>
+      <c r="E18" s="54" t="s">
+        <v>1570</v>
+      </c>
+      <c r="F18" s="46" t="s">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A19" s="50" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B19" s="51" t="s">
+        <v>1454</v>
+      </c>
+      <c r="C19" s="46"/>
+      <c r="D19" s="59" t="s">
+        <v>1499</v>
+      </c>
+      <c r="E19" s="52" t="s">
+        <v>1570</v>
+      </c>
+      <c r="F19" s="46" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A20" s="53" t="s">
+        <v>1575</v>
+      </c>
+      <c r="B20" s="46" t="s">
+        <v>1445</v>
+      </c>
+      <c r="C20" s="46"/>
+      <c r="D20" s="48" t="s">
+        <v>1500</v>
+      </c>
+      <c r="E20" s="54" t="s">
+        <v>1571</v>
+      </c>
+      <c r="F20" s="46" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="24.95" customHeight="1">
+      <c r="A21" s="50" t="s">
+        <v>1576</v>
+      </c>
+      <c r="B21" s="51" t="s">
+        <v>1448</v>
+      </c>
+      <c r="C21" s="51"/>
+      <c r="D21" s="59" t="s">
+        <v>1501</v>
+      </c>
+      <c r="E21" s="52" t="s">
+        <v>1571</v>
+      </c>
+      <c r="F21" s="46" t="s">
+        <v>1579</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="21" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AA1DE75-66A2-4BB5-9D6E-88BAB39F5A48}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
@@ -9056,6 +9838,345 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8628761D-8897-4103-9A07-B5EE77259803}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="9" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.625" style="42" customWidth="1"/>
+    <col min="3" max="3" width="30.625" style="42" customWidth="1"/>
+    <col min="4" max="4" width="20.625" style="42" customWidth="1"/>
+    <col min="5" max="5" width="11.25" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="80" customFormat="1" ht="30" customHeight="1">
+      <c r="A1" s="80" t="s">
+        <v>1790</v>
+      </c>
+      <c r="B1" s="85" t="s">
+        <v>1791</v>
+      </c>
+      <c r="C1" s="85" t="s">
+        <v>1737</v>
+      </c>
+      <c r="D1" s="85" t="s">
+        <v>1738</v>
+      </c>
+      <c r="E1" s="80" t="s">
+        <v>1739</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="28.5">
+      <c r="A2" s="78" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B2" s="86" t="s">
+        <v>1775</v>
+      </c>
+      <c r="C2" s="86" t="s">
+        <v>1776</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>678</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="42.75">
+      <c r="A3" s="82" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B3" s="86" t="s">
+        <v>1775</v>
+      </c>
+      <c r="C3" s="86" t="s">
+        <v>1779</v>
+      </c>
+      <c r="D3" s="87" t="s">
+        <v>1742</v>
+      </c>
+      <c r="E3" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="42.75">
+      <c r="A4" s="81" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B4" s="86" t="s">
+        <v>1778</v>
+      </c>
+      <c r="C4" s="86" t="s">
+        <v>1777</v>
+      </c>
+      <c r="D4" s="87" t="s">
+        <v>1743</v>
+      </c>
+      <c r="E4" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="57">
+      <c r="A5" s="82" t="s">
+        <v>1741</v>
+      </c>
+      <c r="B5" s="87" t="s">
+        <v>1778</v>
+      </c>
+      <c r="C5" s="86" t="s">
+        <v>1780</v>
+      </c>
+      <c r="D5" s="86" t="s">
+        <v>1781</v>
+      </c>
+      <c r="E5" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.5">
+      <c r="A6" s="81" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B6" s="86" t="s">
+        <v>1782</v>
+      </c>
+      <c r="C6" s="86" t="s">
+        <v>1783</v>
+      </c>
+      <c r="D6" s="87" t="s">
+        <v>1744</v>
+      </c>
+      <c r="E6" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="42.75">
+      <c r="A7" s="81" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B7" s="87" t="s">
+        <v>1745</v>
+      </c>
+      <c r="C7" s="86" t="s">
+        <v>1784</v>
+      </c>
+      <c r="D7" s="87" t="s">
+        <v>1746</v>
+      </c>
+      <c r="E7" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="42.75">
+      <c r="A8" s="83" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B8" s="87" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C8" s="86" t="s">
+        <v>1785</v>
+      </c>
+      <c r="D8" s="87" t="s">
+        <v>1748</v>
+      </c>
+      <c r="E8" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="28.5">
+      <c r="A9" s="83" t="s">
+        <v>1789</v>
+      </c>
+      <c r="B9" s="87" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="87" t="s">
+        <v>1749</v>
+      </c>
+      <c r="D9" s="87" t="s">
+        <v>1750</v>
+      </c>
+      <c r="E9" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="42.75">
+      <c r="A10" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B10" s="87" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="87" t="s">
+        <v>1751</v>
+      </c>
+      <c r="D10" s="87" t="s">
+        <v>1752</v>
+      </c>
+      <c r="E10" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="28.5">
+      <c r="A11" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B11" s="87" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C11" s="87" t="s">
+        <v>1754</v>
+      </c>
+      <c r="D11" s="87" t="s">
+        <v>1755</v>
+      </c>
+      <c r="E11" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="24.95" customHeight="1">
+      <c r="A12" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B12" s="87" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C12" s="87" t="s">
+        <v>1757</v>
+      </c>
+      <c r="D12" s="87" t="s">
+        <v>1758</v>
+      </c>
+      <c r="E12" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="28.5">
+      <c r="A13" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B13" s="87" t="s">
+        <v>1759</v>
+      </c>
+      <c r="C13" s="87" t="s">
+        <v>1760</v>
+      </c>
+      <c r="D13" s="87" t="s">
+        <v>1761</v>
+      </c>
+      <c r="E13" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="24.95" customHeight="1">
+      <c r="A14" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B14" s="87" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C14" s="87" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D14" s="87" t="s">
+        <v>1764</v>
+      </c>
+      <c r="E14" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="28.5">
+      <c r="A15" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B15" s="87" t="s">
+        <v>1765</v>
+      </c>
+      <c r="C15" s="87" t="s">
+        <v>1766</v>
+      </c>
+      <c r="D15" s="87" t="s">
+        <v>1767</v>
+      </c>
+      <c r="E15" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="28.5">
+      <c r="A16" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B16" s="87" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C16" s="87" t="s">
+        <v>1769</v>
+      </c>
+      <c r="D16" s="87" t="s">
+        <v>1770</v>
+      </c>
+      <c r="E16" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="85.5">
+      <c r="A17" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B17" s="87" t="s">
+        <v>1771</v>
+      </c>
+      <c r="C17" s="86" t="s">
+        <v>1786</v>
+      </c>
+      <c r="D17" s="87" t="s">
+        <v>1772</v>
+      </c>
+      <c r="E17" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.5">
+      <c r="A18" s="83" t="s">
+        <v>1788</v>
+      </c>
+      <c r="B18" s="87" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C18" s="86" t="s">
+        <v>1787</v>
+      </c>
+      <c r="D18" s="87" t="s">
+        <v>1774</v>
+      </c>
+      <c r="E18" s="82" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="24.95" customHeight="1">
+      <c r="A19" s="84"/>
+      <c r="B19" s="88"/>
+      <c r="C19" s="88"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="84"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E2">
+    <sortCondition ref="A1:A2"/>
+  </sortState>
+  <phoneticPr fontId="32" type="noConversion"/>
+  <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="94" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1832CE4E-6640-4F77-AE2C-2BCFE1960A83}">
   <dimension ref="A1:K445"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -17384,7 +18505,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC2AA81C-8F1F-4458-8028-A2B83F85B815}">
   <dimension ref="A1:F61"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -18558,7 +19679,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06CB5D3A-60EF-41A0-A517-7415BF086DA6}">
   <dimension ref="B1:G17"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="24.95" customHeight="1"/>
@@ -18922,7 +20043,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D004169C-3805-4C15-8A78-8EFBD42CAEA3}">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -18964,7 +20085,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04810001-19A2-4057-9492-DAB102C978CB}">
   <dimension ref="A1:F198"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -23145,7 +24266,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{777D3A3F-8E01-42AE-AC20-239C93F52F98}">
   <dimension ref="A1:F215"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -27469,7 +28590,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C67ABFE6-0E3D-41E3-A8E9-BDC84F153A78}">
   <dimension ref="A1:G236"/>
   <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
@@ -33289,424 +34410,4 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D43CC4C-71E3-46F9-8C94-C607BA6D0756}">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultRowHeight="24.95" customHeight="1"/>
-  <cols>
-    <col min="1" max="1" width="17.25" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.875" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8" style="2" customWidth="1"/>
-    <col min="4" max="4" width="20" style="42" customWidth="1"/>
-    <col min="5" max="5" width="6.625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="18.375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" s="58" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A1" s="55" t="s">
-        <v>1563</v>
-      </c>
-      <c r="B1" s="75" t="s">
-        <v>1726</v>
-      </c>
-      <c r="C1" s="75" t="s">
-        <v>1727</v>
-      </c>
-      <c r="D1" s="56" t="s">
-        <v>1535</v>
-      </c>
-      <c r="E1" s="57" t="s">
-        <v>1536</v>
-      </c>
-      <c r="F1" s="56" t="s">
-        <v>1553</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A2" s="50" t="s">
-        <v>1537</v>
-      </c>
-      <c r="B2" s="51" t="s">
-        <v>1538</v>
-      </c>
-      <c r="C2" s="51" t="s">
-        <v>1516</v>
-      </c>
-      <c r="D2" s="59" t="s">
-        <v>1539</v>
-      </c>
-      <c r="E2" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F2" s="49" t="s">
-        <v>1555</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A3" s="50" t="s">
-        <v>1567</v>
-      </c>
-      <c r="B3" s="51" t="s">
-        <v>1545</v>
-      </c>
-      <c r="C3" s="51" t="s">
-        <v>558</v>
-      </c>
-      <c r="D3" s="59" t="s">
-        <v>1045</v>
-      </c>
-      <c r="E3" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F3" s="49" t="s">
-        <v>1555</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A4" s="50" t="s">
-        <v>1568</v>
-      </c>
-      <c r="B4" s="51" t="s">
-        <v>1546</v>
-      </c>
-      <c r="C4" s="51" t="s">
-        <v>559</v>
-      </c>
-      <c r="D4" s="59" t="s">
-        <v>1046</v>
-      </c>
-      <c r="E4" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F4" s="49" t="s">
-        <v>1555</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="28.5">
-      <c r="A5" s="50" t="s">
-        <v>1569</v>
-      </c>
-      <c r="B5" s="51" t="s">
-        <v>1547</v>
-      </c>
-      <c r="C5" s="51" t="s">
-        <v>1552</v>
-      </c>
-      <c r="D5" s="59" t="s">
-        <v>811</v>
-      </c>
-      <c r="E5" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F5" s="74" t="s">
-        <v>1554</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A6" s="50" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B6" s="51" t="s">
-        <v>1548</v>
-      </c>
-      <c r="C6" s="51" t="s">
-        <v>562</v>
-      </c>
-      <c r="D6" s="59" t="s">
-        <v>1047</v>
-      </c>
-      <c r="E6" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F6" s="46" t="s">
-        <v>1556</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A7" s="50" t="s">
-        <v>1542</v>
-      </c>
-      <c r="B7" s="51" t="s">
-        <v>1549</v>
-      </c>
-      <c r="C7" s="51" t="s">
-        <v>563</v>
-      </c>
-      <c r="D7" s="59" t="s">
-        <v>815</v>
-      </c>
-      <c r="E7" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F7" s="46" t="s">
-        <v>1557</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A8" s="50" t="s">
-        <v>1543</v>
-      </c>
-      <c r="B8" s="51" t="s">
-        <v>1550</v>
-      </c>
-      <c r="C8" s="51" t="s">
-        <v>818</v>
-      </c>
-      <c r="D8" s="59" t="s">
-        <v>817</v>
-      </c>
-      <c r="E8" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F8" s="46" t="s">
-        <v>1558</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="28.5">
-      <c r="A9" s="50" t="s">
-        <v>1544</v>
-      </c>
-      <c r="B9" s="51" t="s">
-        <v>1551</v>
-      </c>
-      <c r="C9" s="51" t="s">
-        <v>564</v>
-      </c>
-      <c r="D9" s="59" t="s">
-        <v>820</v>
-      </c>
-      <c r="E9" s="52" t="s">
-        <v>1540</v>
-      </c>
-      <c r="F9" s="60" t="s">
-        <v>1566</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A10" s="76" t="s">
-        <v>1728</v>
-      </c>
-      <c r="B10" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>1562</v>
-      </c>
-      <c r="D10" s="48" t="s">
-        <v>1048</v>
-      </c>
-      <c r="E10" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F10" s="46"/>
-    </row>
-    <row r="11" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A11" s="53" t="s">
-        <v>1564</v>
-      </c>
-      <c r="B11" s="46" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="46" t="s">
-        <v>571</v>
-      </c>
-      <c r="D11" s="48" t="s">
-        <v>1507</v>
-      </c>
-      <c r="E11" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F11" s="46"/>
-    </row>
-    <row r="12" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A12" s="53" t="s">
-        <v>1565</v>
-      </c>
-      <c r="B12" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="46" t="s">
-        <v>572</v>
-      </c>
-      <c r="D12" s="48" t="s">
-        <v>827</v>
-      </c>
-      <c r="E12" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F12" s="46"/>
-    </row>
-    <row r="13" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A13" s="53" t="s">
-        <v>1559</v>
-      </c>
-      <c r="B13" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="46" t="s">
-        <v>573</v>
-      </c>
-      <c r="D13" s="48" t="s">
-        <v>829</v>
-      </c>
-      <c r="E13" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F13" s="46"/>
-    </row>
-    <row r="14" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A14" s="53" t="s">
-        <v>832</v>
-      </c>
-      <c r="B14" s="46" t="s">
-        <v>69</v>
-      </c>
-      <c r="C14" s="46" t="s">
-        <v>574</v>
-      </c>
-      <c r="D14" s="48" t="s">
-        <v>1480</v>
-      </c>
-      <c r="E14" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F14" s="46"/>
-    </row>
-    <row r="15" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A15" s="53" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>575</v>
-      </c>
-      <c r="D15" s="48" t="s">
-        <v>1481</v>
-      </c>
-      <c r="E15" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F15" s="46"/>
-    </row>
-    <row r="16" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A16" s="53" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" s="46" t="s">
-        <v>89</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>576</v>
-      </c>
-      <c r="D16" s="48" t="s">
-        <v>1482</v>
-      </c>
-      <c r="E16" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F16" s="46"/>
-    </row>
-    <row r="17" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A17" s="50" t="s">
-        <v>1560</v>
-      </c>
-      <c r="B17" s="51" t="s">
-        <v>97</v>
-      </c>
-      <c r="C17" s="46" t="s">
-        <v>577</v>
-      </c>
-      <c r="D17" s="59" t="s">
-        <v>836</v>
-      </c>
-      <c r="E17" s="54" t="s">
-        <v>1561</v>
-      </c>
-      <c r="F17" s="51"/>
-    </row>
-    <row r="18" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A18" s="53" t="s">
-        <v>1573</v>
-      </c>
-      <c r="B18" s="46" t="s">
-        <v>1451</v>
-      </c>
-      <c r="C18" s="46"/>
-      <c r="D18" s="48" t="s">
-        <v>1498</v>
-      </c>
-      <c r="E18" s="54" t="s">
-        <v>1570</v>
-      </c>
-      <c r="F18" s="46" t="s">
-        <v>1572</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A19" s="50" t="s">
-        <v>1574</v>
-      </c>
-      <c r="B19" s="51" t="s">
-        <v>1454</v>
-      </c>
-      <c r="C19" s="46"/>
-      <c r="D19" s="59" t="s">
-        <v>1499</v>
-      </c>
-      <c r="E19" s="52" t="s">
-        <v>1570</v>
-      </c>
-      <c r="F19" s="46" t="s">
-        <v>1577</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A20" s="53" t="s">
-        <v>1575</v>
-      </c>
-      <c r="B20" s="46" t="s">
-        <v>1445</v>
-      </c>
-      <c r="C20" s="46"/>
-      <c r="D20" s="48" t="s">
-        <v>1500</v>
-      </c>
-      <c r="E20" s="54" t="s">
-        <v>1571</v>
-      </c>
-      <c r="F20" s="46" t="s">
-        <v>1578</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="24.95" customHeight="1">
-      <c r="A21" s="50" t="s">
-        <v>1576</v>
-      </c>
-      <c r="B21" s="51" t="s">
-        <v>1448</v>
-      </c>
-      <c r="C21" s="51"/>
-      <c r="D21" s="59" t="s">
-        <v>1501</v>
-      </c>
-      <c r="E21" s="52" t="s">
-        <v>1571</v>
-      </c>
-      <c r="F21" s="46" t="s">
-        <v>1579</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>